<commit_message>
data: actualizar Letras Activas + agregar skill /audit
- Letras Activas.xlsx: actualización de letras vigentes
- .claude/skills/audit/SKILL.md: checklist de auditoría de producción
  (seguridad, filtrado de datos, APIs externas, UI, bugs conocidos)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/Letras Activas.xlsx
+++ b/backend/data/Letras Activas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\.shortcut-targets-by-id\1ftoIZqhxjIK-zxyM2xIG9xFIX4GG9BvJ\DCF\Claude\dcf-herramientas-web\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{357FEDB3-6BB1-41FE-B32B-901CC777F0F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{466F3A29-7448-4B04-A864-EF2CBA571E5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{CD73C5C9-5C4F-49BA-8BAE-0ED83DF77E5D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CD73C5C9-5C4F-49BA-8BAE-0ED83DF77E5D}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>T30J6</t>
   </si>
@@ -99,6 +99,9 @@
   </si>
   <si>
     <t>S12J6</t>
+  </si>
+  <si>
+    <t>S15S6</t>
   </si>
 </sst>
 </file>
@@ -476,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EE54452-AF50-4305-B8DA-DFD46BDACA81}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="17.81640625" style="2" bestFit="1" customWidth="1"/>
@@ -583,78 +586,89 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B10" s="1">
-        <v>46295</v>
+        <v>46280</v>
       </c>
       <c r="C10">
-        <v>117.54</v>
+        <v>107.21</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="B11" s="1">
-        <v>46325</v>
+        <v>46295</v>
       </c>
       <c r="C11">
-        <v>135.28</v>
+        <v>117.54</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B12" s="1">
-        <v>46356</v>
+        <v>46325</v>
       </c>
       <c r="C12">
-        <v>129.88999999999999</v>
+        <v>135.28</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
+      </c>
+      <c r="B13" s="1">
+        <v>46356</v>
       </c>
       <c r="C13">
-        <v>161.1</v>
+        <v>129.88999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="1">
-        <v>46507</v>
+        <v>1</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>8</v>
       </c>
       <c r="C14">
-        <v>157.34</v>
+        <v>161.1</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B15" s="1">
-        <v>46538</v>
+        <v>46507</v>
       </c>
       <c r="C15">
-        <v>151.56</v>
+        <v>157.34</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="1">
+        <v>46538</v>
+      </c>
+      <c r="C16">
+        <v>151.56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B17" s="1">
         <v>46568</v>
       </c>
-      <c r="C16">
+      <c r="C17">
         <v>156.04</v>
       </c>
     </row>

</xml_diff>